<commit_message>
feat Gemini AI generated schedule
</commit_message>
<xml_diff>
--- a/backend/experiments/data/input_schedule.xlsx
+++ b/backend/experiments/data/input_schedule.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E103"/>
+  <dimension ref="A1:E61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -458,12 +458,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Clase_01</t>
+          <t>Clase_001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Prof_82</t>
+          <t>Prof_41</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -485,12 +485,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Clase_02</t>
+          <t>Clase_002</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Prof_32</t>
+          <t>Prof_16</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -512,12 +512,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Clase_03</t>
+          <t>Clase_003</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Prof_87</t>
+          <t>Prof_44</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -539,12 +539,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Clase_04</t>
+          <t>Clase_004</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Prof_05</t>
+          <t>Prof_03</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -566,12 +566,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Clase_05</t>
+          <t>Clase_005</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Prof_65</t>
+          <t>Prof_33</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -593,12 +593,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Clase_06</t>
+          <t>Clase_006</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Prof_92</t>
+          <t>Prof_46</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -620,12 +620,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Clase_07</t>
+          <t>Clase_007</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Prof_76</t>
+          <t>Prof_38</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -647,12 +647,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Clase_08</t>
+          <t>Clase_008</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Prof_55</t>
+          <t>Prof_28</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -674,12 +674,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Clase_09</t>
+          <t>Clase_009</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Prof_98</t>
+          <t>Prof_49</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -701,12 +701,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Clase_10</t>
+          <t>Clase_010</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Prof_13</t>
+          <t>Prof_07</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -728,12 +728,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Clase_11</t>
+          <t>Clase_011</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Prof_06</t>
+          <t>Prof_03</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -755,12 +755,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Clase_12</t>
+          <t>Clase_012</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Prof_11</t>
+          <t>Prof_06</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -782,12 +782,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Clase_13</t>
+          <t>Clase_013</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Prof_47</t>
+          <t>Prof_24</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -809,12 +809,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Clase_14</t>
+          <t>Clase_014</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Prof_06</t>
+          <t>Prof_03</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -836,12 +836,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Clase_15</t>
+          <t>Clase_015</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Prof_13</t>
+          <t>Prof_07</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -863,12 +863,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Clase_16</t>
+          <t>Clase_016</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Prof_47</t>
+          <t>Prof_24</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -890,12 +890,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Clase_17</t>
+          <t>Clase_017</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Prof_86</t>
+          <t>Prof_43</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -917,12 +917,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Clase_18</t>
+          <t>Clase_018</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Prof_10</t>
+          <t>Prof_05</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -944,12 +944,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Clase_19</t>
+          <t>Clase_019</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Prof_94</t>
+          <t>Prof_47</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -971,12 +971,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Clase_20</t>
+          <t>Clase_020</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Prof_35</t>
+          <t>Prof_18</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -998,12 +998,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Clase_21</t>
+          <t>Clase_021</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Prof_99</t>
+          <t>Prof_50</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1025,12 +1025,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Clase_22</t>
+          <t>Clase_022</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Prof_52</t>
+          <t>Prof_26</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1052,12 +1052,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Clase_23</t>
+          <t>Clase_023</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Prof_92</t>
+          <t>Prof_46</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1079,12 +1079,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Clase_24</t>
+          <t>Clase_024</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Prof_51</t>
+          <t>Prof_26</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1106,12 +1106,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Clase_25</t>
+          <t>Clase_025</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Prof_32</t>
+          <t>Prof_16</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1133,12 +1133,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Clase_26</t>
+          <t>Clase_026</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Prof_75</t>
+          <t>Prof_38</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1160,12 +1160,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Clase_27</t>
+          <t>Clase_027</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Prof_29</t>
+          <t>Prof_15</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1187,12 +1187,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Clase_28</t>
+          <t>Clase_028</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Prof_97</t>
+          <t>Prof_49</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1214,12 +1214,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Clase_29</t>
+          <t>Clase_029</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Prof_21</t>
+          <t>Prof_11</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1241,12 +1241,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Clase_30</t>
+          <t>Clase_030</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Prof_49</t>
+          <t>Prof_25</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1268,12 +1268,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Clase_31</t>
+          <t>Clase_031</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Prof_71</t>
+          <t>Prof_36</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1295,12 +1295,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Clase_32</t>
+          <t>Clase_032</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Prof_88</t>
+          <t>Prof_44</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1322,12 +1322,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Clase_33</t>
+          <t>Clase_033</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Prof_15</t>
+          <t>Prof_08</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1349,7 +1349,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Clase_34</t>
+          <t>Clase_034</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1376,12 +1376,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Clase_35</t>
+          <t>Clase_035</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Prof_14</t>
+          <t>Prof_07</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1403,12 +1403,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Clase_36</t>
+          <t>Clase_036</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Prof_26</t>
+          <t>Prof_13</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1430,12 +1430,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Clase_37</t>
+          <t>Clase_037</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Prof_100</t>
+          <t>Prof_50</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1457,12 +1457,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Clase_38</t>
+          <t>Clase_038</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Prof_63</t>
+          <t>Prof_32</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1484,12 +1484,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Clase_39</t>
+          <t>Clase_039</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Prof_31</t>
+          <t>Prof_16</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1511,12 +1511,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Clase_40</t>
+          <t>Clase_040</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Prof_11</t>
+          <t>Prof_06</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1538,12 +1538,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Clase_41</t>
+          <t>Clase_041</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Prof_17</t>
+          <t>Prof_09</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1565,12 +1565,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Clase_42</t>
+          <t>Clase_042</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Prof_68</t>
+          <t>Prof_34</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1592,12 +1592,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Clase_43</t>
+          <t>Clase_043</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Prof_97</t>
+          <t>Prof_49</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1619,12 +1619,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Clase_44</t>
+          <t>Clase_044</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Prof_86</t>
+          <t>Prof_43</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1646,12 +1646,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Clase_45</t>
+          <t>Clase_045</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Prof_16</t>
+          <t>Prof_08</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1673,12 +1673,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Clase_46</t>
+          <t>Clase_046</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Prof_03</t>
+          <t>Prof_02</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -1700,12 +1700,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Clase_47</t>
+          <t>Clase_047</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Prof_29</t>
+          <t>Prof_15</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -1727,12 +1727,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Clase_48</t>
+          <t>Clase_048</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Prof_08</t>
+          <t>Prof_04</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -1754,12 +1754,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Clase_49</t>
+          <t>Clase_049</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Prof_10</t>
+          <t>Prof_05</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -1781,12 +1781,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Clase_50</t>
+          <t>Clase_050</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Prof_63</t>
+          <t>Prof_32</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -1808,12 +1808,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Clase_51</t>
+          <t>Clase_051</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Prof_74</t>
+          <t>Prof_37</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -1835,12 +1835,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Clase_52</t>
+          <t>Clase_052</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Prof_53</t>
+          <t>Prof_27</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -1862,12 +1862,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Clase_53</t>
+          <t>Clase_053</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Prof_56</t>
+          <t>Prof_28</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -1889,12 +1889,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Clase_54</t>
+          <t>Clase_054</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Prof_94</t>
+          <t>Prof_47</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -1916,12 +1916,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Clase_55</t>
+          <t>Clase_055</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Prof_13</t>
+          <t>Prof_07</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -1943,12 +1943,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Clase_56</t>
+          <t>Clase_056</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Prof_14</t>
+          <t>Prof_07</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -1970,12 +1970,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Clase_57</t>
+          <t>Clase_057</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Prof_58</t>
+          <t>Prof_29</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -1997,12 +1997,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Clase_58</t>
+          <t>Clase_058</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Prof_60</t>
+          <t>Prof_30</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2024,12 +2024,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Clase_59</t>
+          <t>Clase_059</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Prof_13</t>
+          <t>Prof_07</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2051,12 +2051,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Clase_60</t>
+          <t>Clase_060</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Prof_12</t>
+          <t>Prof_06</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2072,1140 +2072,6 @@
       <c r="E61" t="inlineStr">
         <is>
           <t>10:00-18:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>Clase_61</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>Prof_62</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>Martes</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>G4</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>07:00-16:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>Clase_62</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>Prof_49</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>Lunes</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>G4</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>09:00-18:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>Clase_63</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>Prof_37</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>Jueves</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>G6</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>12:00-19:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>Clase_64</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>Prof_85</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>Jueves</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>G2</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>08:00-17:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>Clase_65</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>Prof_28</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>Lunes</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>G5</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>12:00-19:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>Clase_66</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>Prof_08</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>Miércoles</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>G1</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>07:00-19:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>Clase_67</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>Prof_62</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>G5</t>
-        </is>
-      </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>08:00-15:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>Clase_68</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>Prof_66</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>Lunes</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>G2</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>07:00-19:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>Clase_69</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>Prof_09</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>Martes</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>G4</t>
-        </is>
-      </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>07:00-19:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>Clase_70</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>Prof_32</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>G5</t>
-        </is>
-      </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>07:00-19:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>Clase_71</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>Prof_11</t>
-        </is>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>Jueves</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>G6</t>
-        </is>
-      </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>11:00-19:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>Clase_72</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>Prof_67</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>Miércoles</t>
-        </is>
-      </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>G3</t>
-        </is>
-      </c>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>08:00-20:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>Clase_73</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>Prof_92</t>
-        </is>
-      </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>Miércoles</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>G2</t>
-        </is>
-      </c>
-      <c r="E74" t="inlineStr">
-        <is>
-          <t>09:00-18:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>Clase_74</t>
-        </is>
-      </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>Prof_17</t>
-        </is>
-      </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>Miércoles</t>
-        </is>
-      </c>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>G4</t>
-        </is>
-      </c>
-      <c r="E75" t="inlineStr">
-        <is>
-          <t>09:00-15:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>Clase_75</t>
-        </is>
-      </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>Prof_02</t>
-        </is>
-      </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>Jueves</t>
-        </is>
-      </c>
-      <c r="D76" t="inlineStr">
-        <is>
-          <t>G5</t>
-        </is>
-      </c>
-      <c r="E76" t="inlineStr">
-        <is>
-          <t>11:00-15:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>Clase_76</t>
-        </is>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>Prof_10</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>G2</t>
-        </is>
-      </c>
-      <c r="E77" t="inlineStr">
-        <is>
-          <t>11:00-17:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="inlineStr">
-        <is>
-          <t>Clase_77</t>
-        </is>
-      </c>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>Prof_17</t>
-        </is>
-      </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>Miércoles</t>
-        </is>
-      </c>
-      <c r="D78" t="inlineStr">
-        <is>
-          <t>G1</t>
-        </is>
-      </c>
-      <c r="E78" t="inlineStr">
-        <is>
-          <t>08:00-17:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t>Clase_78</t>
-        </is>
-      </c>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>Prof_37</t>
-        </is>
-      </c>
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>Martes</t>
-        </is>
-      </c>
-      <c r="D79" t="inlineStr">
-        <is>
-          <t>G4</t>
-        </is>
-      </c>
-      <c r="E79" t="inlineStr">
-        <is>
-          <t>11:00-20:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t>Clase_79</t>
-        </is>
-      </c>
-      <c r="B80" t="inlineStr">
-        <is>
-          <t>Prof_39</t>
-        </is>
-      </c>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="D80" t="inlineStr">
-        <is>
-          <t>G6</t>
-        </is>
-      </c>
-      <c r="E80" t="inlineStr">
-        <is>
-          <t>11:00-15:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t>Clase_80</t>
-        </is>
-      </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>Prof_86</t>
-        </is>
-      </c>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="D81" t="inlineStr">
-        <is>
-          <t>G3</t>
-        </is>
-      </c>
-      <c r="E81" t="inlineStr">
-        <is>
-          <t>12:00-15:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="inlineStr">
-        <is>
-          <t>Clase_81</t>
-        </is>
-      </c>
-      <c r="B82" t="inlineStr">
-        <is>
-          <t>Prof_18</t>
-        </is>
-      </c>
-      <c r="C82" t="inlineStr">
-        <is>
-          <t>Miércoles</t>
-        </is>
-      </c>
-      <c r="D82" t="inlineStr">
-        <is>
-          <t>G1</t>
-        </is>
-      </c>
-      <c r="E82" t="inlineStr">
-        <is>
-          <t>07:00-20:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" t="inlineStr">
-        <is>
-          <t>Clase_82</t>
-        </is>
-      </c>
-      <c r="B83" t="inlineStr">
-        <is>
-          <t>Prof_71</t>
-        </is>
-      </c>
-      <c r="C83" t="inlineStr">
-        <is>
-          <t>Martes</t>
-        </is>
-      </c>
-      <c r="D83" t="inlineStr">
-        <is>
-          <t>G3</t>
-        </is>
-      </c>
-      <c r="E83" t="inlineStr">
-        <is>
-          <t>09:00-19:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t>Clase_83</t>
-        </is>
-      </c>
-      <c r="B84" t="inlineStr">
-        <is>
-          <t>Prof_27</t>
-        </is>
-      </c>
-      <c r="C84" t="inlineStr">
-        <is>
-          <t>Miércoles</t>
-        </is>
-      </c>
-      <c r="D84" t="inlineStr">
-        <is>
-          <t>G2</t>
-        </is>
-      </c>
-      <c r="E84" t="inlineStr">
-        <is>
-          <t>12:00-20:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" t="inlineStr">
-        <is>
-          <t>Clase_84</t>
-        </is>
-      </c>
-      <c r="B85" t="inlineStr">
-        <is>
-          <t>Prof_34</t>
-        </is>
-      </c>
-      <c r="C85" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="D85" t="inlineStr">
-        <is>
-          <t>G4</t>
-        </is>
-      </c>
-      <c r="E85" t="inlineStr">
-        <is>
-          <t>09:00-15:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" t="inlineStr">
-        <is>
-          <t>Clase_85</t>
-        </is>
-      </c>
-      <c r="B86" t="inlineStr">
-        <is>
-          <t>Prof_12</t>
-        </is>
-      </c>
-      <c r="C86" t="inlineStr">
-        <is>
-          <t>Jueves</t>
-        </is>
-      </c>
-      <c r="D86" t="inlineStr">
-        <is>
-          <t>G3</t>
-        </is>
-      </c>
-      <c r="E86" t="inlineStr">
-        <is>
-          <t>07:00-15:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" t="inlineStr">
-        <is>
-          <t>Clase_86</t>
-        </is>
-      </c>
-      <c r="B87" t="inlineStr">
-        <is>
-          <t>Prof_43</t>
-        </is>
-      </c>
-      <c r="C87" t="inlineStr">
-        <is>
-          <t>Martes</t>
-        </is>
-      </c>
-      <c r="D87" t="inlineStr">
-        <is>
-          <t>G6</t>
-        </is>
-      </c>
-      <c r="E87" t="inlineStr">
-        <is>
-          <t>09:00-16:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t>Clase_87</t>
-        </is>
-      </c>
-      <c r="B88" t="inlineStr">
-        <is>
-          <t>Prof_95</t>
-        </is>
-      </c>
-      <c r="C88" t="inlineStr">
-        <is>
-          <t>Jueves</t>
-        </is>
-      </c>
-      <c r="D88" t="inlineStr">
-        <is>
-          <t>G5</t>
-        </is>
-      </c>
-      <c r="E88" t="inlineStr">
-        <is>
-          <t>12:00-18:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" t="inlineStr">
-        <is>
-          <t>Clase_88</t>
-        </is>
-      </c>
-      <c r="B89" t="inlineStr">
-        <is>
-          <t>Prof_72</t>
-        </is>
-      </c>
-      <c r="C89" t="inlineStr">
-        <is>
-          <t>Lunes</t>
-        </is>
-      </c>
-      <c r="D89" t="inlineStr">
-        <is>
-          <t>G1</t>
-        </is>
-      </c>
-      <c r="E89" t="inlineStr">
-        <is>
-          <t>07:00-20:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" t="inlineStr">
-        <is>
-          <t>Clase_89</t>
-        </is>
-      </c>
-      <c r="B90" t="inlineStr">
-        <is>
-          <t>Prof_20</t>
-        </is>
-      </c>
-      <c r="C90" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="D90" t="inlineStr">
-        <is>
-          <t>G1</t>
-        </is>
-      </c>
-      <c r="E90" t="inlineStr">
-        <is>
-          <t>09:00-19:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" t="inlineStr">
-        <is>
-          <t>Clase_90</t>
-        </is>
-      </c>
-      <c r="B91" t="inlineStr">
-        <is>
-          <t>Prof_71</t>
-        </is>
-      </c>
-      <c r="C91" t="inlineStr">
-        <is>
-          <t>Martes</t>
-        </is>
-      </c>
-      <c r="D91" t="inlineStr">
-        <is>
-          <t>G4</t>
-        </is>
-      </c>
-      <c r="E91" t="inlineStr">
-        <is>
-          <t>08:00-15:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" t="inlineStr">
-        <is>
-          <t>Clase_91</t>
-        </is>
-      </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>Prof_40</t>
-        </is>
-      </c>
-      <c r="C92" t="inlineStr">
-        <is>
-          <t>Miércoles</t>
-        </is>
-      </c>
-      <c r="D92" t="inlineStr">
-        <is>
-          <t>G1</t>
-        </is>
-      </c>
-      <c r="E92" t="inlineStr">
-        <is>
-          <t>09:00-16:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="inlineStr">
-        <is>
-          <t>Clase_92</t>
-        </is>
-      </c>
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>Prof_88</t>
-        </is>
-      </c>
-      <c r="C93" t="inlineStr">
-        <is>
-          <t>Martes</t>
-        </is>
-      </c>
-      <c r="D93" t="inlineStr">
-        <is>
-          <t>G6</t>
-        </is>
-      </c>
-      <c r="E93" t="inlineStr">
-        <is>
-          <t>07:00-17:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" t="inlineStr">
-        <is>
-          <t>Clase_93</t>
-        </is>
-      </c>
-      <c r="B94" t="inlineStr">
-        <is>
-          <t>Prof_100</t>
-        </is>
-      </c>
-      <c r="C94" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="D94" t="inlineStr">
-        <is>
-          <t>G4</t>
-        </is>
-      </c>
-      <c r="E94" t="inlineStr">
-        <is>
-          <t>11:00-20:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" t="inlineStr">
-        <is>
-          <t>Clase_94</t>
-        </is>
-      </c>
-      <c r="B95" t="inlineStr">
-        <is>
-          <t>Prof_20</t>
-        </is>
-      </c>
-      <c r="C95" t="inlineStr">
-        <is>
-          <t>Martes</t>
-        </is>
-      </c>
-      <c r="D95" t="inlineStr">
-        <is>
-          <t>G2</t>
-        </is>
-      </c>
-      <c r="E95" t="inlineStr">
-        <is>
-          <t>08:00-18:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" t="inlineStr">
-        <is>
-          <t>Clase_95</t>
-        </is>
-      </c>
-      <c r="B96" t="inlineStr">
-        <is>
-          <t>Prof_04</t>
-        </is>
-      </c>
-      <c r="C96" t="inlineStr">
-        <is>
-          <t>Martes</t>
-        </is>
-      </c>
-      <c r="D96" t="inlineStr">
-        <is>
-          <t>G6</t>
-        </is>
-      </c>
-      <c r="E96" t="inlineStr">
-        <is>
-          <t>09:00-18:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="inlineStr">
-        <is>
-          <t>Clase_96</t>
-        </is>
-      </c>
-      <c r="B97" t="inlineStr">
-        <is>
-          <t>Prof_86</t>
-        </is>
-      </c>
-      <c r="C97" t="inlineStr">
-        <is>
-          <t>Martes</t>
-        </is>
-      </c>
-      <c r="D97" t="inlineStr">
-        <is>
-          <t>G3</t>
-        </is>
-      </c>
-      <c r="E97" t="inlineStr">
-        <is>
-          <t>08:00-20:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="inlineStr">
-        <is>
-          <t>Clase_97</t>
-        </is>
-      </c>
-      <c r="B98" t="inlineStr">
-        <is>
-          <t>Prof_14</t>
-        </is>
-      </c>
-      <c r="C98" t="inlineStr">
-        <is>
-          <t>Jueves</t>
-        </is>
-      </c>
-      <c r="D98" t="inlineStr">
-        <is>
-          <t>G1</t>
-        </is>
-      </c>
-      <c r="E98" t="inlineStr">
-        <is>
-          <t>10:00-16:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" t="inlineStr">
-        <is>
-          <t>Clase_98</t>
-        </is>
-      </c>
-      <c r="B99" t="inlineStr">
-        <is>
-          <t>Prof_26</t>
-        </is>
-      </c>
-      <c r="C99" t="inlineStr">
-        <is>
-          <t>Jueves</t>
-        </is>
-      </c>
-      <c r="D99" t="inlineStr">
-        <is>
-          <t>G3</t>
-        </is>
-      </c>
-      <c r="E99" t="inlineStr">
-        <is>
-          <t>09:00-16:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" t="inlineStr">
-        <is>
-          <t>Clase_99</t>
-        </is>
-      </c>
-      <c r="B100" t="inlineStr">
-        <is>
-          <t>Prof_29</t>
-        </is>
-      </c>
-      <c r="C100" t="inlineStr">
-        <is>
-          <t>Lunes</t>
-        </is>
-      </c>
-      <c r="D100" t="inlineStr">
-        <is>
-          <t>G6</t>
-        </is>
-      </c>
-      <c r="E100" t="inlineStr">
-        <is>
-          <t>08:00-18:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" t="inlineStr">
-        <is>
-          <t>Clase_100</t>
-        </is>
-      </c>
-      <c r="B101" t="inlineStr">
-        <is>
-          <t>Prof_43</t>
-        </is>
-      </c>
-      <c r="C101" t="inlineStr">
-        <is>
-          <t>Miércoles</t>
-        </is>
-      </c>
-      <c r="D101" t="inlineStr">
-        <is>
-          <t>G1</t>
-        </is>
-      </c>
-      <c r="E101" t="inlineStr">
-        <is>
-          <t>09:00-17:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" t="inlineStr">
-        <is>
-          <t>Clase_101</t>
-        </is>
-      </c>
-      <c r="B102" t="inlineStr">
-        <is>
-          <t>Prof_83</t>
-        </is>
-      </c>
-      <c r="C102" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="D102" t="inlineStr">
-        <is>
-          <t>G4</t>
-        </is>
-      </c>
-      <c r="E102" t="inlineStr">
-        <is>
-          <t>12:00-19:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" t="inlineStr">
-        <is>
-          <t>Clase_102</t>
-        </is>
-      </c>
-      <c r="B103" t="inlineStr">
-        <is>
-          <t>Prof_43</t>
-        </is>
-      </c>
-      <c r="C103" t="inlineStr">
-        <is>
-          <t>Lunes</t>
-        </is>
-      </c>
-      <c r="D103" t="inlineStr">
-        <is>
-          <t>G1</t>
-        </is>
-      </c>
-      <c r="E103" t="inlineStr">
-        <is>
-          <t>09:00-16:00</t>
         </is>
       </c>
     </row>

</xml_diff>